<commit_message>
fix(reimbursements): stop the BACS template naming a budget holder
The vendored authorisation form carried a fixed name and designation, so any
cost centre without its own printed them. Those two cells are now blank with
their styling kept; every other part of the workbook is byte-identical.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/lib/reimbursements/templates/EUSA_BACS_template.xlsx
+++ b/lib/reimbursements/templates/EUSA_BACS_template.xlsx
@@ -65,7 +65,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56" count="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56" count="54">
   <si>
     <t>BANK PAYMENT INTERNAL BULK REQUEST</t>
   </si>
@@ -165,7 +165,7 @@
     <t>NAME</t>
   </si>
   <si>
-    <t>Mick Zijdel</t>
+    <t/>
   </si>
   <si>
     <t>SIGNATURE</t>
@@ -174,7 +174,7 @@
     <t>DESIGNATION</t>
   </si>
   <si>
-    <t>Bedlam Fringe Production Manager</t>
+    <t/>
   </si>
   <si>
     <t>DATE</t>
@@ -1308,9 +1308,7 @@
       <c r="B16" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="19" t="s">
-        <v>17</v>
-      </c>
+      <c r="C16" s="19"/>
       <c r="D16" s="18" t="s">
         <v>18</v>
       </c>
@@ -1320,9 +1318,7 @@
       <c r="B17" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="22" t="s">
-        <v>20</v>
-      </c>
+      <c r="C17" s="22"/>
       <c r="D17" s="23" t="s">
         <v>21</v>
       </c>

</xml_diff>